<commit_message>
Renewal FRS comparison: BDOI's technical words shown in business words, new annex letters after Z, corrected counts and quotes
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Comparisons/BIBS_Comparison_BRD-06_BDOI_FRS_vs_BIBS_FRS_Renewal_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Comparisons/BIBS_Comparison_BRD-06_BDOI_FRS_vs_BIBS_FRS_Renewal_v1.0.xlsx
@@ -5963,7 +5963,7 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Same: 13, Partial: 57, Different: 18, Not in ours: 55</t>
+          <t>Same: 12, Partial: 58, Different: 18, Not in ours: 55</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr"/>
@@ -60906,7 +60906,7 @@
       </c>
       <c r="G71" s="29" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="H71" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Renewal FRS comparison: a conflict is to confirm only where the BIBS FRS follows the BRD or the platform; the others are for BDOI to decide
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Comparisons/BIBS_Comparison_BRD-06_BDOI_FRS_vs_BIBS_FRS_Renewal_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Comparisons/BIBS_Comparison_BRD-06_BDOI_FRS_vs_BIBS_FRS_Renewal_v1.0.xlsx
@@ -1594,7 +1594,7 @@
       </c>
       <c r="I8" s="29" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>Decide</t>
         </is>
       </c>
       <c r="J8" s="12" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="I9" s="29" t="inlineStr">
         <is>
-          <t>Confirm</t>
+          <t>Decide</t>
         </is>
       </c>
       <c r="J9" s="12" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Only in ours: 43 items; conflicting: 28 points, of which 17 where the BIBS FRS follows the BRD or the platform</t>
+          <t>Only in ours: 43 items; conflicting: 28 points, of which 15 where the BIBS FRS follows the BRD or the platform</t>
         </is>
       </c>
     </row>

</xml_diff>